<commit_message>
feat(masterdata): 판치기 타격 커널 노브
</commit_message>
<xml_diff>
--- a/table/Datas/#PanchigiConfig.xlsx
+++ b/table/Datas/#PanchigiConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,31 @@
           <t>drop_out_limit</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>force_multiplier</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>horizontal_force_multiplier</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>falloff_rate</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>coverage_samples</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>hold_time_max</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -509,6 +534,31 @@
           <t>int</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -561,6 +611,31 @@
       <c r="I4" t="inlineStr">
         <is>
           <t>drop_out_limit</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>force_multiplier</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>horizontal_force_multiplier</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>falloff_rate</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>coverage_samples</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>hold_time_max</t>
         </is>
       </c>
     </row>
@@ -588,6 +663,21 @@
       </c>
       <c r="I5" t="n">
         <v>3</v>
+      </c>
+      <c r="J5" t="n">
+        <v>40</v>
+      </c>
+      <c r="K5" t="n">
+        <v>20</v>
+      </c>
+      <c r="L5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M5" t="n">
+        <v>13</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(masterdata): 판치기 접촉점 상한(contact_max) 컬럼을 넣는다
</commit_message>
<xml_diff>
--- a/table/Datas/#PanchigiConfig.xlsx
+++ b/table/Datas/#PanchigiConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,6 +487,11 @@
           <t>hold_time_max</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>contact_max</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -559,6 +564,11 @@
           <t>float</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -636,6 +646,11 @@
       <c r="N4" t="inlineStr">
         <is>
           <t>hold_time_max</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>contact_max</t>
         </is>
       </c>
     </row>
@@ -678,6 +693,9 @@
       </c>
       <c r="N5" t="n">
         <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>